<commit_message>
[Etapa 6] Canasta comparable, conclusiones finales y actualización del README
</commit_message>
<xml_diff>
--- a/data/processed/productos_etiquetados_parcialmente.xlsx
+++ b/data/processed/productos_etiquetados_parcialmente.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nesto\Desktop\Github\analisis-precios-NLP-SEPA\data\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C3ACF6F-A87D-4E1A-B58D-265895DDD917}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0FF9A42-5FED-4FA1-B736-3A5674C2DCBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -14344,11 +14344,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EE8A8A95-9171-4298-8F33-CA16F23C5312}" name="Tabla1" displayName="Tabla1" ref="A1:G2221" totalsRowShown="0">
-  <autoFilter ref="A1:G2221" xr:uid="{EE8A8A95-9171-4298-8F33-CA16F23C5312}">
-    <filterColumn colId="6">
-      <filters blank="1"/>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:G2221" xr:uid="{EE8A8A95-9171-4298-8F33-CA16F23C5312}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{695A9560-60AA-441D-9491-4ACBFE73B5B3}" name="id_producto"/>
     <tableColumn id="2" xr3:uid="{59DA3F1B-7D81-4437-BBAA-D850E0AEB8FA}" name="precio_medio_carrefour"/>
@@ -14682,7 +14678,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>40084107</v>
       </c>
@@ -14765,7 +14761,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>75083694</v>
       </c>
@@ -14808,7 +14804,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>77903785</v>
       </c>
@@ -14851,7 +14847,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>77907943</v>
       </c>
@@ -14874,7 +14870,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>77908308</v>
       </c>
@@ -14897,7 +14893,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>77908377</v>
       </c>
@@ -14920,7 +14916,7 @@
         <v>4702</v>
       </c>
     </row>
-    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>77927361</v>
       </c>
@@ -14943,7 +14939,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>77949677</v>
       </c>
@@ -14966,7 +14962,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>77953124</v>
       </c>
@@ -14989,7 +14985,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>77956262</v>
       </c>
@@ -15012,7 +15008,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>77973986</v>
       </c>
@@ -15035,7 +15031,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>77976109</v>
       </c>
@@ -15058,7 +15054,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>77988263</v>
       </c>
@@ -15081,7 +15077,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>77991577</v>
       </c>
@@ -15104,7 +15100,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>77991584</v>
       </c>
@@ -15127,7 +15123,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>78600010</v>
       </c>
@@ -15170,7 +15166,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>78909434</v>
       </c>
@@ -15193,7 +15189,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>78923454</v>
       </c>
@@ -15296,7 +15292,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>80052487</v>
       </c>
@@ -15319,7 +15315,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>80052760</v>
       </c>
@@ -15382,7 +15378,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>90435225</v>
       </c>
@@ -15405,7 +15401,7 @@
         <v>4702</v>
       </c>
     </row>
-    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>41333001005</v>
       </c>
@@ -15428,7 +15424,7 @@
         <v>4712</v>
       </c>
     </row>
-    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>41333001029</v>
       </c>
@@ -15451,7 +15447,7 @@
         <v>4712</v>
       </c>
     </row>
-    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>41333001074</v>
       </c>
@@ -15474,7 +15470,7 @@
         <v>4712</v>
       </c>
     </row>
-    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>41333001098</v>
       </c>
@@ -15517,7 +15513,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>70330734395</v>
       </c>
@@ -15560,7 +15556,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>70942005500</v>
       </c>
@@ -15603,7 +15599,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>70942306805</v>
       </c>
@@ -15686,7 +15682,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>608875008994</v>
       </c>
@@ -15709,7 +15705,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>650240035401</v>
       </c>
@@ -15732,7 +15728,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>650240051647</v>
       </c>
@@ -15755,7 +15751,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>650240069352</v>
       </c>
@@ -15918,7 +15914,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>4005808524105</v>
       </c>
@@ -16041,7 +16037,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>4005900036759</v>
       </c>
@@ -16124,7 +16120,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>4005900717238</v>
       </c>
@@ -16167,7 +16163,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>4005900806161</v>
       </c>
@@ -16230,7 +16226,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="74" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>4006000005478</v>
       </c>
@@ -16333,7 +16329,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>4006000195681</v>
       </c>
@@ -16436,7 +16432,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="84" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>5000267014005</v>
       </c>
@@ -16459,7 +16455,7 @@
         <v>4702</v>
       </c>
     </row>
-    <row r="85" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>5000281015248</v>
       </c>
@@ -16482,7 +16478,7 @@
         <v>4702</v>
       </c>
     </row>
-    <row r="86" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>5900273001566</v>
       </c>
@@ -16505,7 +16501,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="87" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>6001298008123</v>
       </c>
@@ -16528,7 +16524,7 @@
         <v>4712</v>
       </c>
     </row>
-    <row r="88" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>6001495062508</v>
       </c>
@@ -16551,7 +16547,7 @@
         <v>4702</v>
       </c>
     </row>
-    <row r="89" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>7312040017683</v>
       </c>
@@ -16574,7 +16570,7 @@
         <v>4702</v>
       </c>
     </row>
-    <row r="90" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>7500435019880</v>
       </c>
@@ -16697,7 +16693,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="96" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>7500435150248</v>
       </c>
@@ -16780,7 +16776,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="100" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>7500435160087</v>
       </c>
@@ -16803,7 +16799,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="101" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>7500435169646</v>
       </c>
@@ -17066,7 +17062,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="114" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>7500435225366</v>
       </c>
@@ -17089,7 +17085,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="115" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>7500435228572</v>
       </c>
@@ -17252,7 +17248,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="123" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>7500435229579</v>
       </c>
@@ -17375,7 +17371,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="129" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>7500435233019</v>
       </c>
@@ -17518,7 +17514,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="136" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>7500435242677</v>
       </c>
@@ -17581,7 +17577,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="139" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>7500435243674</v>
       </c>
@@ -17844,7 +17840,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="152" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>7500810034477</v>
       </c>
@@ -17867,7 +17863,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="153" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>7500810041734</v>
       </c>
@@ -17930,7 +17926,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="156" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>7501054542896</v>
       </c>
@@ -17953,7 +17949,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="157" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>7501058753441</v>
       </c>
@@ -17976,7 +17972,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="158" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>7501058753458</v>
       </c>
@@ -18239,7 +18235,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="171" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>7506339332643</v>
       </c>
@@ -18302,7 +18298,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="174" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>7509546070988</v>
       </c>
@@ -18405,7 +18401,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="179" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>7509546679617</v>
       </c>
@@ -18448,7 +18444,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="181" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>7509546683393</v>
       </c>
@@ -18531,7 +18527,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="185" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>7509546686523</v>
       </c>
@@ -18614,7 +18610,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="189" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>7509546688145</v>
       </c>
@@ -18737,7 +18733,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="195" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>7509546703640</v>
       </c>
@@ -19200,7 +19196,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="218" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>7509552923759</v>
       </c>
@@ -19503,7 +19499,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="233" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>7509552979558</v>
       </c>
@@ -19546,7 +19542,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="235" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>7613287149145</v>
       </c>
@@ -19569,7 +19565,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="236" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>7613287225191</v>
       </c>
@@ -19592,7 +19588,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="237" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>7613287229977</v>
       </c>
@@ -19615,7 +19611,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="238" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>7613287230386</v>
       </c>
@@ -19638,7 +19634,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="239" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>7613287613226</v>
       </c>
@@ -19661,7 +19657,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="240" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>7613287613240</v>
       </c>
@@ -19684,7 +19680,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="241" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>7613287613356</v>
       </c>
@@ -19727,7 +19723,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="243" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>7613287613455</v>
       </c>
@@ -19750,7 +19746,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="244" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>7613287614971</v>
       </c>
@@ -19773,7 +19769,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="245" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>7622201492465</v>
       </c>
@@ -19916,7 +19912,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="252" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>7622201703059</v>
       </c>
@@ -19999,7 +19995,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="256" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>7622201703172</v>
       </c>
@@ -20042,7 +20038,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="258" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>7622201705961</v>
       </c>
@@ -20065,7 +20061,7 @@
         <v>4702</v>
       </c>
     </row>
-    <row r="259" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>7622201705992</v>
       </c>
@@ -20088,7 +20084,7 @@
         <v>4702</v>
       </c>
     </row>
-    <row r="260" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>7622201733865</v>
       </c>
@@ -20131,7 +20127,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="262" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>7622201735296</v>
       </c>
@@ -20214,7 +20210,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="266" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A266">
         <v>7622201735715</v>
       </c>
@@ -20317,7 +20313,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="271" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A271">
         <v>7622201736033</v>
       </c>
@@ -20400,7 +20396,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="275" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A275">
         <v>7622201745967</v>
       </c>
@@ -20583,7 +20579,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="284" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A284">
         <v>7622202247316</v>
       </c>
@@ -20646,7 +20642,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="287" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A287">
         <v>7622202304705</v>
       </c>
@@ -20749,7 +20745,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="292" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A292">
         <v>7622202816437</v>
       </c>
@@ -20912,7 +20908,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="300" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A300">
         <v>7630040411011</v>
       </c>
@@ -21035,7 +21031,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="306" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A306">
         <v>7702018037865</v>
       </c>
@@ -21078,7 +21074,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="308" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A308">
         <v>7702018072408</v>
       </c>
@@ -21181,7 +21177,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="313" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A313">
         <v>7702103751416</v>
       </c>
@@ -21224,7 +21220,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="315" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A315">
         <v>7702425808041</v>
       </c>
@@ -21247,7 +21243,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="316" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A316">
         <v>7702626214825</v>
       </c>
@@ -21270,7 +21266,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="317" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A317">
         <v>7702626219912</v>
       </c>
@@ -21433,7 +21429,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="325" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A325">
         <v>7790010002929</v>
       </c>
@@ -21496,7 +21492,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="328" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A328">
         <v>7790010003162</v>
       </c>
@@ -21519,7 +21515,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="329" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A329">
         <v>7790010003261</v>
       </c>
@@ -21542,7 +21538,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="330" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A330">
         <v>7790015104109</v>
       </c>
@@ -21625,7 +21621,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="334" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A334">
         <v>7790033338197</v>
       </c>
@@ -21808,7 +21804,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="343" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A343">
         <v>7790040008175</v>
       </c>
@@ -22631,7 +22627,7 @@
         <v>807</v>
       </c>
     </row>
-    <row r="384" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A384">
         <v>7790040148840</v>
       </c>
@@ -22754,7 +22750,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="390" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A390">
         <v>7790045000624</v>
       </c>
@@ -22817,7 +22813,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="393" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A393">
         <v>7790045826965</v>
       </c>
@@ -22840,7 +22836,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="394" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A394">
         <v>7790060023684</v>
       </c>
@@ -22883,7 +22879,7 @@
         <v>905</v>
       </c>
     </row>
-    <row r="396" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A396">
         <v>7790064000261</v>
       </c>
@@ -22906,7 +22902,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="397" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A397">
         <v>7790064001909</v>
       </c>
@@ -22989,7 +22985,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="401" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A401">
         <v>7790070034410</v>
       </c>
@@ -23012,7 +23008,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="402" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A402">
         <v>7790070034427</v>
       </c>
@@ -23035,7 +23031,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="403" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A403">
         <v>7790070035936</v>
       </c>
@@ -23098,7 +23094,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="406" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A406">
         <v>7790070035981</v>
       </c>
@@ -23161,7 +23157,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="409" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A409">
         <v>7790070036278</v>
       </c>
@@ -23224,7 +23220,7 @@
         <v>922</v>
       </c>
     </row>
-    <row r="412" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A412">
         <v>7790070040015</v>
       </c>
@@ -23247,7 +23243,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="413" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A413">
         <v>7790070040039</v>
       </c>
@@ -23270,7 +23266,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="414" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A414">
         <v>7790070100757</v>
       </c>
@@ -23293,7 +23289,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="415" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A415">
         <v>7790070103918</v>
       </c>
@@ -23336,7 +23332,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="417" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A417">
         <v>7790070231864</v>
       </c>
@@ -23399,7 +23395,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="420" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="420" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A420">
         <v>7790070317452</v>
       </c>
@@ -23442,7 +23438,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="422" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="422" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A422">
         <v>7790070318398</v>
       </c>
@@ -23465,7 +23461,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="423" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="423" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A423">
         <v>7790070320001</v>
       </c>
@@ -23488,7 +23484,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="424" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="424" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A424">
         <v>7790070320285</v>
       </c>
@@ -23571,7 +23567,7 @@
         <v>969</v>
       </c>
     </row>
-    <row r="428" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="428" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A428">
         <v>7790070320940</v>
       </c>
@@ -23654,7 +23650,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="432" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="432" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A432">
         <v>7790070335340</v>
       </c>
@@ -23997,7 +23993,7 @@
         <v>987</v>
       </c>
     </row>
-    <row r="449" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="449" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A449">
         <v>7790070336965</v>
       </c>
@@ -24020,7 +24016,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="450" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="450" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A450">
         <v>7790070410801</v>
       </c>
@@ -24103,7 +24099,7 @@
         <v>1028</v>
       </c>
     </row>
-    <row r="454" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="454" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A454">
         <v>7790070412126</v>
       </c>
@@ -24146,7 +24142,7 @@
         <v>1031</v>
       </c>
     </row>
-    <row r="456" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="456" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A456">
         <v>7790070413116</v>
       </c>
@@ -24209,7 +24205,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="459" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="459" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A459">
         <v>7790070417954</v>
       </c>
@@ -24232,7 +24228,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="460" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="460" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A460">
         <v>7790070418203</v>
       </c>
@@ -24315,7 +24311,7 @@
         <v>1023</v>
       </c>
     </row>
-    <row r="464" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="464" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A464">
         <v>7790070431431</v>
       </c>
@@ -24638,7 +24634,7 @@
         <v>1023</v>
       </c>
     </row>
-    <row r="480" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="480" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A480">
         <v>7790070433169</v>
       </c>
@@ -24701,7 +24697,7 @@
         <v>1082</v>
       </c>
     </row>
-    <row r="483" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="483" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A483">
         <v>7790070433244</v>
       </c>
@@ -24784,7 +24780,7 @@
         <v>1095</v>
       </c>
     </row>
-    <row r="487" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="487" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A487">
         <v>7790070507280</v>
       </c>
@@ -24827,7 +24823,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="489" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="489" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A489">
         <v>7790070507372</v>
       </c>
@@ -25010,7 +25006,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="498" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="498" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A498">
         <v>7790070562074</v>
       </c>
@@ -25093,7 +25089,7 @@
         <v>969</v>
       </c>
     </row>
-    <row r="502" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="502" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A502">
         <v>7790070562265</v>
       </c>
@@ -25136,7 +25132,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="504" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="504" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A504">
         <v>7790070621863</v>
       </c>
@@ -25199,7 +25195,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="507" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="507" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A507">
         <v>7790070622020</v>
       </c>
@@ -25302,7 +25298,7 @@
         <v>1150</v>
       </c>
     </row>
-    <row r="512" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="512" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A512">
         <v>7790070760562</v>
       </c>
@@ -25425,7 +25421,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="518" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="518" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A518">
         <v>7790070760760</v>
       </c>
@@ -25528,7 +25524,7 @@
         <v>1169</v>
       </c>
     </row>
-    <row r="523" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="523" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A523">
         <v>7790070764041</v>
       </c>
@@ -25591,7 +25587,7 @@
         <v>1177</v>
       </c>
     </row>
-    <row r="526" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="526" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A526">
         <v>7790071090330</v>
       </c>
@@ -25654,7 +25650,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="529" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="529" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A529">
         <v>7790072001038</v>
       </c>
@@ -25697,7 +25693,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="531" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="531" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A531">
         <v>7790079000638</v>
       </c>
@@ -25720,7 +25716,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="532" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="532" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A532">
         <v>7790079001031</v>
       </c>
@@ -25763,7 +25759,7 @@
         <v>1190</v>
       </c>
     </row>
-    <row r="534" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="534" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A534">
         <v>7790079019562</v>
       </c>
@@ -25886,7 +25882,7 @@
         <v>1209</v>
       </c>
     </row>
-    <row r="540" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="540" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A540">
         <v>7790130000034</v>
       </c>
@@ -25929,7 +25925,7 @@
         <v>1209</v>
       </c>
     </row>
-    <row r="542" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="542" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A542">
         <v>7790132009158</v>
       </c>
@@ -25952,7 +25948,7 @@
         <v>4712</v>
       </c>
     </row>
-    <row r="543" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="543" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A543">
         <v>7790132098459</v>
       </c>
@@ -25975,7 +25971,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="544" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="544" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A544">
         <v>7790139002879</v>
       </c>
@@ -26078,7 +26074,7 @@
         <v>1224</v>
       </c>
     </row>
-    <row r="549" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="549" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A549">
         <v>7790150101476</v>
       </c>
@@ -26201,7 +26197,7 @@
         <v>1224</v>
       </c>
     </row>
-    <row r="555" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="555" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A555">
         <v>7790150310267</v>
       </c>
@@ -26324,7 +26320,7 @@
         <v>1253</v>
       </c>
     </row>
-    <row r="561" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="561" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A561">
         <v>7790150435380</v>
       </c>
@@ -26447,7 +26443,7 @@
         <v>1253</v>
       </c>
     </row>
-    <row r="567" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="567" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A567">
         <v>7790150490334</v>
       </c>
@@ -26670,7 +26666,7 @@
         <v>1288</v>
       </c>
     </row>
-    <row r="578" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="578" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A578">
         <v>7790154000829</v>
       </c>
@@ -26753,7 +26749,7 @@
         <v>1297</v>
       </c>
     </row>
-    <row r="582" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="582" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A582">
         <v>7790154008306</v>
       </c>
@@ -26816,7 +26812,7 @@
         <v>1297</v>
       </c>
     </row>
-    <row r="585" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="585" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A585">
         <v>7790158229547</v>
       </c>
@@ -26939,7 +26935,7 @@
         <v>1309</v>
       </c>
     </row>
-    <row r="591" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="591" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A591">
         <v>7790170903654</v>
       </c>
@@ -27002,7 +26998,7 @@
         <v>1309</v>
       </c>
     </row>
-    <row r="594" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="594" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A594">
         <v>7790174001318</v>
       </c>
@@ -27065,7 +27061,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="597" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="597" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A597">
         <v>7790174001417</v>
       </c>
@@ -27168,7 +27164,7 @@
         <v>1337</v>
       </c>
     </row>
-    <row r="602" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="602" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A602">
         <v>7790197120218</v>
       </c>
@@ -27351,7 +27347,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="611" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="611" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A611">
         <v>7790199604587</v>
       </c>
@@ -27454,7 +27450,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="616" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="616" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A616">
         <v>7790236018353</v>
       </c>
@@ -27757,7 +27753,7 @@
         <v>1398</v>
       </c>
     </row>
-    <row r="631" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="631" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A631">
         <v>7790250015840</v>
       </c>
@@ -27900,7 +27896,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="638" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="638" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A638">
         <v>7790250042068</v>
       </c>
@@ -27983,7 +27979,7 @@
         <v>1409</v>
       </c>
     </row>
-    <row r="642" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="642" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A642">
         <v>7790250056881</v>
       </c>
@@ -28006,7 +28002,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="643" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="643" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A643">
         <v>7790250057086</v>
       </c>
@@ -28089,7 +28085,7 @@
         <v>1432</v>
       </c>
     </row>
-    <row r="647" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="647" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A647">
         <v>7790250097624</v>
       </c>
@@ -28212,7 +28208,7 @@
         <v>1443</v>
       </c>
     </row>
-    <row r="653" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="653" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A653">
         <v>7790290001179</v>
       </c>
@@ -28235,7 +28231,7 @@
         <v>4702</v>
       </c>
     </row>
-    <row r="654" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="654" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A654">
         <v>7790290008192</v>
       </c>
@@ -28378,7 +28374,7 @@
         <v>1466</v>
       </c>
     </row>
-    <row r="661" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="661" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A661">
         <v>7790310983270</v>
       </c>
@@ -28401,7 +28397,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="662" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="662" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A662">
         <v>7790310983553</v>
       </c>
@@ -28444,7 +28440,7 @@
         <v>1474</v>
       </c>
     </row>
-    <row r="664" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="664" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A664">
         <v>7790310984321</v>
       </c>
@@ -28527,7 +28523,7 @@
         <v>1484</v>
       </c>
     </row>
-    <row r="668" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="668" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A668">
         <v>7790310985137</v>
       </c>
@@ -28850,7 +28846,7 @@
         <v>1491</v>
       </c>
     </row>
-    <row r="684" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="684" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A684">
         <v>7790310985649</v>
       </c>
@@ -29213,7 +29209,7 @@
         <v>1550</v>
       </c>
     </row>
-    <row r="702" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="702" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A702">
         <v>7790314079726</v>
       </c>
@@ -29356,7 +29352,7 @@
         <v>1563</v>
       </c>
     </row>
-    <row r="709" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="709" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A709">
         <v>7790314080166</v>
       </c>
@@ -29419,7 +29415,7 @@
         <v>1555</v>
       </c>
     </row>
-    <row r="712" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="712" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A712">
         <v>7790314081279</v>
       </c>
@@ -29462,7 +29458,7 @@
         <v>1573</v>
       </c>
     </row>
-    <row r="714" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="714" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A714">
         <v>7790315000880</v>
       </c>
@@ -29525,7 +29521,7 @@
         <v>1581</v>
       </c>
     </row>
-    <row r="717" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="717" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A717">
         <v>7790360026590</v>
       </c>
@@ -29568,7 +29564,7 @@
         <v>1581</v>
       </c>
     </row>
-    <row r="719" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="719" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A719">
         <v>7790360720115</v>
       </c>
@@ -29591,7 +29587,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="720" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="720" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A720">
         <v>7790360720382</v>
       </c>
@@ -29614,7 +29610,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="721" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="721" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A721">
         <v>7790360966841</v>
       </c>
@@ -29697,7 +29693,7 @@
         <v>1581</v>
       </c>
     </row>
-    <row r="725" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="725" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A725">
         <v>7790360983947</v>
       </c>
@@ -29780,7 +29776,7 @@
         <v>1605</v>
       </c>
     </row>
-    <row r="729" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="729" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A729">
         <v>7790380258018</v>
       </c>
@@ -29983,7 +29979,7 @@
         <v>1612</v>
       </c>
     </row>
-    <row r="739" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="739" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A739">
         <v>7790387800135</v>
       </c>
@@ -30046,7 +30042,7 @@
         <v>1634</v>
       </c>
     </row>
-    <row r="742" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="742" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A742">
         <v>7790398100088</v>
       </c>
@@ -30089,7 +30085,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="744" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="744" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A744">
         <v>7790398100132</v>
       </c>
@@ -30212,7 +30208,7 @@
         <v>1646</v>
       </c>
     </row>
-    <row r="750" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="750" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A750">
         <v>7790416066532</v>
       </c>
@@ -30335,7 +30331,7 @@
         <v>1664</v>
       </c>
     </row>
-    <row r="756" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="756" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A756">
         <v>7790480089765</v>
       </c>
@@ -30378,7 +30374,7 @@
         <v>1664</v>
       </c>
     </row>
-    <row r="758" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="758" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A758">
         <v>7790480090006</v>
       </c>
@@ -30461,7 +30457,7 @@
         <v>1676</v>
       </c>
     </row>
-    <row r="762" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="762" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A762">
         <v>7790490998064</v>
       </c>
@@ -30484,7 +30480,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="763" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="763" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A763">
         <v>7790490998231</v>
       </c>
@@ -30527,7 +30523,7 @@
         <v>1676</v>
       </c>
     </row>
-    <row r="765" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="765" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A765">
         <v>7790520014863</v>
       </c>
@@ -30550,7 +30546,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="766" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="766" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A766">
         <v>7790520018618</v>
       </c>
@@ -30593,7 +30589,7 @@
         <v>1692</v>
       </c>
     </row>
-    <row r="768" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="768" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A768">
         <v>7790520025722</v>
       </c>
@@ -30616,7 +30612,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="769" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="769" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A769">
         <v>7790520025753</v>
       </c>
@@ -30639,7 +30635,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="770" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="770" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A770">
         <v>7790520025777</v>
       </c>
@@ -30662,7 +30658,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="771" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="771" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A771">
         <v>7790520025869</v>
       </c>
@@ -30685,7 +30681,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="772" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="772" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A772">
         <v>7790520026132</v>
       </c>
@@ -30708,7 +30704,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="773" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="773" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A773">
         <v>7790520026170</v>
       </c>
@@ -30751,7 +30747,7 @@
         <v>1692</v>
       </c>
     </row>
-    <row r="775" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="775" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A775">
         <v>7790520028082</v>
       </c>
@@ -30794,7 +30790,7 @@
         <v>1712</v>
       </c>
     </row>
-    <row r="777" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="777" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A777">
         <v>7790520028556</v>
       </c>
@@ -30817,7 +30813,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="778" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="778" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A778">
         <v>7790520028648</v>
       </c>
@@ -30840,7 +30836,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="779" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="779" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A779">
         <v>7790520028747</v>
       </c>
@@ -30863,7 +30859,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="780" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="780" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A780">
         <v>7790520028877</v>
       </c>
@@ -30886,7 +30882,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="781" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="781" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A781">
         <v>7790520028914</v>
       </c>
@@ -30969,7 +30965,7 @@
         <v>1712</v>
       </c>
     </row>
-    <row r="785" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="785" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A785">
         <v>7790520031426</v>
       </c>
@@ -30992,7 +30988,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="786" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="786" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A786">
         <v>7790520031570</v>
       </c>
@@ -31035,7 +31031,7 @@
         <v>1692</v>
       </c>
     </row>
-    <row r="788" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="788" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A788">
         <v>7790520989956</v>
       </c>
@@ -31058,7 +31054,7 @@
         <v>4712</v>
       </c>
     </row>
-    <row r="789" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="789" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A789">
         <v>7790520995285</v>
       </c>
@@ -31181,7 +31177,7 @@
         <v>1752</v>
       </c>
     </row>
-    <row r="795" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="795" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A795">
         <v>7790520995971</v>
       </c>
@@ -31224,7 +31220,7 @@
         <v>1727</v>
       </c>
     </row>
-    <row r="797" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="797" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A797">
         <v>7790520996053</v>
       </c>
@@ -31307,7 +31303,7 @@
         <v>1692</v>
       </c>
     </row>
-    <row r="801" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="801" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A801">
         <v>7790520997678</v>
       </c>
@@ -31350,7 +31346,7 @@
         <v>1727</v>
       </c>
     </row>
-    <row r="803" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="803" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A803">
         <v>7790520998279</v>
       </c>
@@ -31393,7 +31389,7 @@
         <v>1689</v>
       </c>
     </row>
-    <row r="805" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="805" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A805">
         <v>7790520998880</v>
       </c>
@@ -31636,7 +31632,7 @@
         <v>1794</v>
       </c>
     </row>
-    <row r="817" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="817" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A817">
         <v>7790580056001</v>
       </c>
@@ -31699,7 +31695,7 @@
         <v>1643</v>
       </c>
     </row>
-    <row r="820" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="820" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A820">
         <v>7790580121303</v>
       </c>
@@ -31742,7 +31738,7 @@
         <v>1809</v>
       </c>
     </row>
-    <row r="822" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="822" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A822">
         <v>7790580124557</v>
       </c>
@@ -31765,7 +31761,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="823" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="823" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A823">
         <v>7790580129606</v>
       </c>
@@ -31808,7 +31804,7 @@
         <v>1819</v>
       </c>
     </row>
-    <row r="825" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="825" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A825">
         <v>7790580131364</v>
       </c>
@@ -31931,7 +31927,7 @@
         <v>1809</v>
       </c>
     </row>
-    <row r="831" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="831" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A831">
         <v>7790580132187</v>
       </c>
@@ -32014,7 +32010,7 @@
         <v>1809</v>
       </c>
     </row>
-    <row r="835" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="835" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A835">
         <v>7790580132255</v>
       </c>
@@ -32117,7 +32113,7 @@
         <v>878</v>
       </c>
     </row>
-    <row r="840" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="840" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A840">
         <v>7790580134341</v>
       </c>
@@ -32140,7 +32136,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="841" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="841" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A841">
         <v>7790580138721</v>
       </c>
@@ -32163,7 +32159,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="842" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="842" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A842">
         <v>7790580138738</v>
       </c>
@@ -32206,7 +32202,7 @@
         <v>1819</v>
       </c>
     </row>
-    <row r="844" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="844" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A844">
         <v>7790580140434</v>
       </c>
@@ -32229,7 +32225,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="845" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="845" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A845">
         <v>7790580141844</v>
       </c>
@@ -32412,7 +32408,7 @@
         <v>1809</v>
       </c>
     </row>
-    <row r="854" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="854" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A854">
         <v>7790580155025</v>
       </c>
@@ -32475,7 +32471,7 @@
         <v>878</v>
       </c>
     </row>
-    <row r="857" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="857" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A857">
         <v>7790580504410</v>
       </c>
@@ -32538,7 +32534,7 @@
         <v>1809</v>
       </c>
     </row>
-    <row r="860" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="860" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A860">
         <v>7790580567903</v>
       </c>
@@ -32561,7 +32557,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="861" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="861" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A861">
         <v>7790580602000</v>
       </c>
@@ -32644,7 +32640,7 @@
         <v>1898</v>
       </c>
     </row>
-    <row r="865" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="865" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A865">
         <v>7790625000303</v>
       </c>
@@ -32707,7 +32703,7 @@
         <v>1903</v>
       </c>
     </row>
-    <row r="868" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="868" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A868">
         <v>7790625005292</v>
       </c>
@@ -32750,7 +32746,7 @@
         <v>1903</v>
       </c>
     </row>
-    <row r="870" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="870" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A870">
         <v>7790625005353</v>
       </c>
@@ -32793,7 +32789,7 @@
         <v>1903</v>
       </c>
     </row>
-    <row r="872" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="872" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A872">
         <v>7790625010296</v>
       </c>
@@ -32816,7 +32812,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="873" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="873" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A873">
         <v>7790625010401</v>
       </c>
@@ -32859,7 +32855,7 @@
         <v>1924</v>
       </c>
     </row>
-    <row r="875" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="875" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A875">
         <v>7790670050667</v>
       </c>
@@ -33142,7 +33138,7 @@
         <v>1956</v>
       </c>
     </row>
-    <row r="889" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="889" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A889">
         <v>7790740000264</v>
       </c>
@@ -33365,7 +33361,7 @@
         <v>1983</v>
       </c>
     </row>
-    <row r="900" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="900" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A900">
         <v>7790742141101</v>
       </c>
@@ -33408,7 +33404,7 @@
         <v>1976</v>
       </c>
     </row>
-    <row r="902" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="902" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A902">
         <v>7790742141606</v>
       </c>
@@ -33451,7 +33447,7 @@
         <v>1976</v>
       </c>
     </row>
-    <row r="904" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="904" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A904">
         <v>7790742172105</v>
       </c>
@@ -33614,7 +33610,7 @@
         <v>2006</v>
       </c>
     </row>
-    <row r="912" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="912" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A912">
         <v>7790742321800</v>
       </c>
@@ -33997,7 +33993,7 @@
         <v>2039</v>
       </c>
     </row>
-    <row r="931" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="931" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A931">
         <v>7790742436207</v>
       </c>
@@ -34060,7 +34056,7 @@
         <v>1976</v>
       </c>
     </row>
-    <row r="934" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="934" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A934">
         <v>7790742625205</v>
       </c>
@@ -34243,7 +34239,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="943" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="943" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A943">
         <v>7790773034014</v>
       </c>
@@ -34306,7 +34302,7 @@
         <v>2072</v>
       </c>
     </row>
-    <row r="946" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="946" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A946">
         <v>7790787030132</v>
       </c>
@@ -34389,7 +34385,7 @@
         <v>2072</v>
       </c>
     </row>
-    <row r="950" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="950" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A950">
         <v>7790787960651</v>
       </c>
@@ -34432,7 +34428,7 @@
         <v>2072</v>
       </c>
     </row>
-    <row r="952" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="952" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A952">
         <v>7790787960934</v>
       </c>
@@ -34495,7 +34491,7 @@
         <v>2087</v>
       </c>
     </row>
-    <row r="955" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="955" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A955">
         <v>7790813150131</v>
       </c>
@@ -34518,7 +34514,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="956" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="956" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A956">
         <v>7790813444469</v>
       </c>
@@ -34541,7 +34537,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="957" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="957" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A957">
         <v>7790813900989</v>
       </c>
@@ -34784,7 +34780,7 @@
         <v>2120</v>
       </c>
     </row>
-    <row r="969" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="969" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A969">
         <v>7790895006036</v>
       </c>
@@ -35067,7 +35063,7 @@
         <v>2148</v>
       </c>
     </row>
-    <row r="983" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="983" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A983">
         <v>7790895643842</v>
       </c>
@@ -35110,7 +35106,7 @@
         <v>2148</v>
       </c>
     </row>
-    <row r="985" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="985" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A985">
         <v>7790895647017</v>
       </c>
@@ -35533,7 +35529,7 @@
         <v>2173</v>
       </c>
     </row>
-    <row r="1006" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1006" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1006">
         <v>7790950142921</v>
       </c>
@@ -35636,7 +35632,7 @@
         <v>2208</v>
       </c>
     </row>
-    <row r="1011" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1011" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1011">
         <v>7790975198859</v>
       </c>
@@ -35739,7 +35735,7 @@
         <v>1956</v>
       </c>
     </row>
-    <row r="1016" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1016" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1016">
         <v>7790990002834</v>
       </c>
@@ -35762,7 +35758,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="1017" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1017" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1017">
         <v>7790990002964</v>
       </c>
@@ -35825,7 +35821,7 @@
         <v>2227</v>
       </c>
     </row>
-    <row r="1020" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1020" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1020">
         <v>7790990003046</v>
       </c>
@@ -35888,7 +35884,7 @@
         <v>2221</v>
       </c>
     </row>
-    <row r="1023" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1023" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1023">
         <v>7790990003220</v>
       </c>
@@ -35911,7 +35907,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="1024" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1024" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1024">
         <v>7790990003787</v>
       </c>
@@ -36474,7 +36470,7 @@
         <v>2264</v>
       </c>
     </row>
-    <row r="1052" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1052" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1052">
         <v>7791130001212</v>
       </c>
@@ -36497,7 +36493,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="1053" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1053" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1053">
         <v>7791130001649</v>
       </c>
@@ -36520,7 +36516,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="1054" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1054" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1054">
         <v>7791130001748</v>
       </c>
@@ -36623,7 +36619,7 @@
         <v>2303</v>
       </c>
     </row>
-    <row r="1059" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1059" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1059">
         <v>7791130146791</v>
       </c>
@@ -36666,7 +36662,7 @@
         <v>2303</v>
       </c>
     </row>
-    <row r="1061" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1061" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1061">
         <v>7791130681384</v>
       </c>
@@ -36749,7 +36745,7 @@
         <v>2303</v>
       </c>
     </row>
-    <row r="1065" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1065" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1065">
         <v>7791130683753</v>
       </c>
@@ -37052,7 +37048,7 @@
         <v>2348</v>
       </c>
     </row>
-    <row r="1080" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1080" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1080">
         <v>7791203003341</v>
       </c>
@@ -37075,7 +37071,7 @@
         <v>4702</v>
       </c>
     </row>
-    <row r="1081" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1081" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1081">
         <v>7791203003396</v>
       </c>
@@ -37198,7 +37194,7 @@
         <v>2365</v>
       </c>
     </row>
-    <row r="1087" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1087" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1087">
         <v>7791250001857</v>
       </c>
@@ -37281,7 +37277,7 @@
         <v>2363</v>
       </c>
     </row>
-    <row r="1091" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1091" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1091">
         <v>7791250003127</v>
       </c>
@@ -37384,7 +37380,7 @@
         <v>2363</v>
       </c>
     </row>
-    <row r="1096" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1096" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1096">
         <v>7791250801532</v>
       </c>
@@ -37447,7 +37443,7 @@
         <v>2391</v>
       </c>
     </row>
-    <row r="1099" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1099" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1099">
         <v>7791290792012</v>
       </c>
@@ -37610,7 +37606,7 @@
         <v>2407</v>
       </c>
     </row>
-    <row r="1107" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1107" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1107">
         <v>7791290792791</v>
       </c>
@@ -37693,7 +37689,7 @@
         <v>2407</v>
       </c>
     </row>
-    <row r="1111" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1111" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1111">
         <v>7791290793354</v>
       </c>
@@ -37716,7 +37712,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="1112" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1112" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1112">
         <v>7791290793361</v>
       </c>
@@ -37779,7 +37775,7 @@
         <v>2426</v>
       </c>
     </row>
-    <row r="1115" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1115" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1115">
         <v>7791290793613</v>
       </c>
@@ -37882,7 +37878,7 @@
         <v>2437</v>
       </c>
     </row>
-    <row r="1120" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1120" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1120">
         <v>7791290794061</v>
       </c>
@@ -37945,7 +37941,7 @@
         <v>2437</v>
       </c>
     </row>
-    <row r="1123" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1123" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1123">
         <v>7791290794092</v>
       </c>
@@ -38008,7 +38004,7 @@
         <v>2437</v>
       </c>
     </row>
-    <row r="1126" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1126" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1126">
         <v>7791290794146</v>
       </c>
@@ -38111,7 +38107,7 @@
         <v>2400</v>
       </c>
     </row>
-    <row r="1131" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1131" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1131">
         <v>7791290794283</v>
       </c>
@@ -38734,7 +38730,7 @@
         <v>2522</v>
       </c>
     </row>
-    <row r="1162" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1162" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1162">
         <v>7791290796669</v>
       </c>
@@ -40857,7 +40853,7 @@
         <v>2585</v>
       </c>
     </row>
-    <row r="1268" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1268" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1268">
         <v>7791293051482</v>
       </c>
@@ -41100,7 +41096,7 @@
         <v>2760</v>
       </c>
     </row>
-    <row r="1280" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1280" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1280">
         <v>7791337007246</v>
       </c>
@@ -41223,7 +41219,7 @@
         <v>2760</v>
       </c>
     </row>
-    <row r="1286" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1286" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1286">
         <v>7791337007802</v>
       </c>
@@ -41446,7 +41442,7 @@
         <v>2800</v>
       </c>
     </row>
-    <row r="1297" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1297" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1297">
         <v>7791337008472</v>
       </c>
@@ -41489,7 +41485,7 @@
         <v>2800</v>
       </c>
     </row>
-    <row r="1299" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1299" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1299">
         <v>7791337008564</v>
       </c>
@@ -41572,7 +41568,7 @@
         <v>2814</v>
       </c>
     </row>
-    <row r="1303" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1303" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1303">
         <v>7791337008663</v>
       </c>
@@ -42315,7 +42311,7 @@
         <v>1976</v>
       </c>
     </row>
-    <row r="1340" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1340" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1340">
         <v>7791337010338</v>
       </c>
@@ -42638,7 +42634,7 @@
         <v>2786</v>
       </c>
     </row>
-    <row r="1356" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1356" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1356">
         <v>7791337010598</v>
       </c>
@@ -42961,7 +42957,7 @@
         <v>1976</v>
       </c>
     </row>
-    <row r="1372" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1372" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1372">
         <v>7791337061491</v>
       </c>
@@ -43104,7 +43100,7 @@
         <v>2955</v>
       </c>
     </row>
-    <row r="1379" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1379" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1379">
         <v>7791540044502</v>
       </c>
@@ -43407,7 +43403,7 @@
         <v>2978</v>
       </c>
     </row>
-    <row r="1394" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1394" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1394">
         <v>7791620187662</v>
       </c>
@@ -43510,7 +43506,7 @@
         <v>2992</v>
       </c>
     </row>
-    <row r="1399" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1399" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1399">
         <v>7791620187778</v>
       </c>
@@ -43593,7 +43589,7 @@
         <v>3009</v>
       </c>
     </row>
-    <row r="1403" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1403" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1403">
         <v>7791670027604</v>
       </c>
@@ -43636,7 +43632,7 @@
         <v>3015</v>
       </c>
     </row>
-    <row r="1405" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1405" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1405">
         <v>7791675909554</v>
       </c>
@@ -43679,7 +43675,7 @@
         <v>3015</v>
       </c>
     </row>
-    <row r="1407" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1407" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1407">
         <v>7791675909684</v>
       </c>
@@ -43902,7 +43898,7 @@
         <v>3042</v>
       </c>
     </row>
-    <row r="1418" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1418" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1418">
         <v>7791813422389</v>
       </c>
@@ -44028,7 +44024,7 @@
         <v>3058</v>
       </c>
     </row>
-    <row r="1424" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1424" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1424">
         <v>7791813444411</v>
       </c>
@@ -44111,7 +44107,7 @@
         <v>3042</v>
       </c>
     </row>
-    <row r="1428" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1428" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1428">
         <v>7791813828365</v>
       </c>
@@ -44214,7 +44210,7 @@
         <v>3075</v>
       </c>
     </row>
-    <row r="1433" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1433" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1433">
         <v>7791813888406</v>
       </c>
@@ -44377,7 +44373,7 @@
         <v>3089</v>
       </c>
     </row>
-    <row r="1441" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1441" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1441">
         <v>7791843009116</v>
       </c>
@@ -44580,7 +44576,7 @@
         <v>1443</v>
       </c>
     </row>
-    <row r="1451" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1451" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1451">
         <v>7791866001357</v>
       </c>
@@ -44875,7 +44871,7 @@
         <v>4702</v>
       </c>
     </row>
-    <row r="1465" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1465" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1465">
         <v>7792170555499</v>
       </c>
@@ -45138,7 +45134,7 @@
         <v>3159</v>
       </c>
     </row>
-    <row r="1478" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1478" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1478">
         <v>7792180131560</v>
       </c>
@@ -45221,7 +45217,7 @@
         <v>1918</v>
       </c>
     </row>
-    <row r="1482" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1482" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1482">
         <v>7792180133465</v>
       </c>
@@ -45644,7 +45640,7 @@
         <v>3205</v>
       </c>
     </row>
-    <row r="1503" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1503" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1503">
         <v>7792180142955</v>
       </c>
@@ -45707,7 +45703,7 @@
         <v>3205</v>
       </c>
     </row>
-    <row r="1506" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1506" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1506">
         <v>7792180145314</v>
       </c>
@@ -45810,7 +45806,7 @@
         <v>3159</v>
       </c>
     </row>
-    <row r="1511" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1511" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1511">
         <v>7792180146397</v>
       </c>
@@ -45833,7 +45829,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="1512" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1512" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1512">
         <v>7792184003085</v>
       </c>
@@ -46196,7 +46192,7 @@
         <v>3272</v>
       </c>
     </row>
-    <row r="1530" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1530" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1530">
         <v>7792390620786</v>
       </c>
@@ -46399,7 +46395,7 @@
         <v>3295</v>
       </c>
     </row>
-    <row r="1540" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1540" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1540">
         <v>7792540250450</v>
       </c>
@@ -46842,7 +46838,7 @@
         <v>3345</v>
       </c>
     </row>
-    <row r="1562" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1562" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1562">
         <v>7792798007493</v>
       </c>
@@ -47068,7 +47064,7 @@
         <v>3338</v>
       </c>
     </row>
-    <row r="1573" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1573" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1573">
         <v>7792798014835</v>
       </c>
@@ -47611,7 +47607,7 @@
         <v>3413</v>
       </c>
     </row>
-    <row r="1600" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1600" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1600">
         <v>7793147570606</v>
       </c>
@@ -47694,7 +47690,7 @@
         <v>3416</v>
       </c>
     </row>
-    <row r="1604" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1604" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1604">
         <v>7793147571689</v>
       </c>
@@ -47737,7 +47733,7 @@
         <v>3410</v>
       </c>
     </row>
-    <row r="1606" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1606" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1606">
         <v>7793147572853</v>
       </c>
@@ -47820,7 +47816,7 @@
         <v>3437</v>
       </c>
     </row>
-    <row r="1610" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1610" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1610">
         <v>7793147574093</v>
       </c>
@@ -48023,7 +48019,7 @@
         <v>3460</v>
       </c>
     </row>
-    <row r="1620" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1620" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1620">
         <v>7793253003722</v>
       </c>
@@ -48086,7 +48082,7 @@
         <v>1218</v>
       </c>
     </row>
-    <row r="1623" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1623" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1623">
         <v>7793253003791</v>
       </c>
@@ -48489,7 +48485,7 @@
         <v>3444</v>
       </c>
     </row>
-    <row r="1643" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1643" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1643">
         <v>7793253007102</v>
       </c>
@@ -48552,7 +48548,7 @@
         <v>3509</v>
       </c>
     </row>
-    <row r="1646" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1646" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1646">
         <v>7793253098773</v>
       </c>
@@ -48655,7 +48651,7 @@
         <v>3522</v>
       </c>
     </row>
-    <row r="1651" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1651" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1651">
         <v>7793281493489</v>
       </c>
@@ -48958,7 +48954,7 @@
         <v>1869</v>
       </c>
     </row>
-    <row r="1666" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1666" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1666">
         <v>7793360132384</v>
       </c>
@@ -49101,7 +49097,7 @@
         <v>3565</v>
       </c>
     </row>
-    <row r="1673" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1673" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1673">
         <v>7793890258264</v>
       </c>
@@ -49184,7 +49180,7 @@
         <v>3575</v>
       </c>
     </row>
-    <row r="1677" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1677" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1677">
         <v>7793890258769</v>
       </c>
@@ -49307,7 +49303,7 @@
         <v>3586</v>
       </c>
     </row>
-    <row r="1683" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1683" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1683">
         <v>7793890258875</v>
       </c>
@@ -49390,7 +49386,7 @@
         <v>3594</v>
       </c>
     </row>
-    <row r="1687" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1687" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1687">
         <v>7793890260724</v>
       </c>
@@ -49493,7 +49489,7 @@
         <v>3586</v>
       </c>
     </row>
-    <row r="1692" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1692" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1692">
         <v>7793890261837</v>
       </c>
@@ -49976,7 +49972,7 @@
         <v>1976</v>
       </c>
     </row>
-    <row r="1716" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1716" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1716">
         <v>7794000004887</v>
       </c>
@@ -50279,7 +50275,7 @@
         <v>3654</v>
       </c>
     </row>
-    <row r="1731" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1731" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1731">
         <v>7794000006164</v>
       </c>
@@ -50382,7 +50378,7 @@
         <v>3691</v>
       </c>
     </row>
-    <row r="1736" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1736" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1736">
         <v>7794000006485</v>
       </c>
@@ -50705,7 +50701,7 @@
         <v>3654</v>
       </c>
     </row>
-    <row r="1752" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1752" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1752">
         <v>7794000008533</v>
       </c>
@@ -51148,7 +51144,7 @@
         <v>3755</v>
       </c>
     </row>
-    <row r="1774" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1774" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1774">
         <v>7794440005109</v>
       </c>
@@ -51251,7 +51247,7 @@
         <v>3755</v>
       </c>
     </row>
-    <row r="1779" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1779" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1779">
         <v>7794440707034</v>
       </c>
@@ -51274,7 +51270,7 @@
         <v>4715</v>
       </c>
     </row>
-    <row r="1780" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1780" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1780">
         <v>7794440994205</v>
       </c>
@@ -51877,7 +51873,7 @@
         <v>3846</v>
       </c>
     </row>
-    <row r="1810" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1810" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1810">
         <v>7794640171741</v>
       </c>
@@ -52920,7 +52916,7 @@
         <v>3946</v>
       </c>
     </row>
-    <row r="1862" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1862" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1862">
         <v>7797394001265</v>
       </c>
@@ -52963,7 +52959,7 @@
         <v>3951</v>
       </c>
     </row>
-    <row r="1864" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1864" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1864">
         <v>7797906054819</v>
       </c>
@@ -53006,7 +53002,7 @@
         <v>3951</v>
       </c>
     </row>
-    <row r="1866" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1866" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1866">
         <v>7797906054864</v>
       </c>
@@ -53089,7 +53085,7 @@
         <v>3965</v>
       </c>
     </row>
-    <row r="1870" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1870" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1870">
         <v>7797906055144</v>
       </c>
@@ -53292,7 +53288,7 @@
         <v>3983</v>
       </c>
     </row>
-    <row r="1880" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1880" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1880">
         <v>7798013103377</v>
       </c>
@@ -53835,7 +53831,7 @@
         <v>1576</v>
       </c>
     </row>
-    <row r="1907" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1907" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1907">
         <v>7798068288128</v>
       </c>
@@ -53858,7 +53854,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="1908" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1908" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1908">
         <v>7798070861401</v>
       </c>
@@ -54141,7 +54137,7 @@
         <v>4054</v>
       </c>
     </row>
-    <row r="1922" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1922" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1922">
         <v>7798104180959</v>
       </c>
@@ -54164,7 +54160,7 @@
         <v>4712</v>
       </c>
     </row>
-    <row r="1923" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1923" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1923">
         <v>7798104180980</v>
       </c>
@@ -54267,7 +54263,7 @@
         <v>4067</v>
       </c>
     </row>
-    <row r="1928" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1928" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1928">
         <v>7798114470057</v>
       </c>
@@ -54290,7 +54286,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="1929" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1929" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1929">
         <v>7798114470194</v>
       </c>
@@ -54333,7 +54329,7 @@
         <v>4076</v>
       </c>
     </row>
-    <row r="1931" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1931" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1931">
         <v>7798119220183</v>
       </c>
@@ -54496,7 +54492,7 @@
         <v>4086</v>
       </c>
     </row>
-    <row r="1939" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1939" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1939">
         <v>7798124362359</v>
       </c>
@@ -54719,7 +54715,7 @@
         <v>1918</v>
       </c>
     </row>
-    <row r="1950" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1950" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1950">
         <v>7798140251712</v>
       </c>
@@ -54962,7 +54958,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="1962" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1962" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1962">
         <v>7798143355608</v>
       </c>
@@ -55065,7 +55061,7 @@
         <v>4153</v>
       </c>
     </row>
-    <row r="1967" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1967" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1967">
         <v>7798151812025</v>
       </c>
@@ -55088,7 +55084,7 @@
         <v>4712</v>
       </c>
     </row>
-    <row r="1968" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1968" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1968">
         <v>7798151952332</v>
       </c>
@@ -55391,7 +55387,7 @@
         <v>4193</v>
       </c>
     </row>
-    <row r="1983" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1983" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1983">
         <v>7798187760857</v>
       </c>
@@ -55474,7 +55470,7 @@
         <v>1616</v>
       </c>
     </row>
-    <row r="1987" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1987" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1987">
         <v>7798262020036</v>
       </c>
@@ -55617,7 +55613,7 @@
         <v>4211</v>
       </c>
     </row>
-    <row r="1994" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1994" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1994">
         <v>7798304840844</v>
       </c>
@@ -55860,7 +55856,7 @@
         <v>4247</v>
       </c>
     </row>
-    <row r="2006" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2006" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2006">
         <v>7798316700815</v>
       </c>
@@ -56283,7 +56279,7 @@
         <v>4296</v>
       </c>
     </row>
-    <row r="2027" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2027" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2027">
         <v>7798342151513</v>
       </c>
@@ -56386,7 +56382,7 @@
         <v>4306</v>
       </c>
     </row>
-    <row r="2032" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2032" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2032">
         <v>7798343751422</v>
       </c>
@@ -56469,7 +56465,7 @@
         <v>4316</v>
       </c>
     </row>
-    <row r="2036" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2036" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2036">
         <v>7798353194721</v>
       </c>
@@ -56712,7 +56708,7 @@
         <v>4338</v>
       </c>
     </row>
-    <row r="2048" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2048" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2048">
         <v>7798456650124</v>
       </c>
@@ -57035,7 +57031,7 @@
         <v>3367</v>
       </c>
     </row>
-    <row r="2064" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2064" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2064">
         <v>7891000120774</v>
       </c>
@@ -57078,7 +57074,7 @@
         <v>4375</v>
       </c>
     </row>
-    <row r="2066" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2066" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2066">
         <v>7891000241134</v>
       </c>
@@ -57101,7 +57097,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="2067" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2067" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2067">
         <v>7891000244012</v>
       </c>
@@ -57124,7 +57120,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="2068" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2068" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2068">
         <v>7891000244036</v>
       </c>
@@ -57147,7 +57143,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="2069" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2069" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2069">
         <v>7891000244074</v>
       </c>
@@ -57450,7 +57446,7 @@
         <v>4411</v>
       </c>
     </row>
-    <row r="2084" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2084" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2084">
         <v>7891010255237</v>
       </c>
@@ -57553,7 +57549,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="2089" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2089" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2089">
         <v>7891010560737</v>
       </c>
@@ -57816,7 +57812,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="2102" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2102" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2102">
         <v>7891024112861</v>
       </c>
@@ -57999,7 +57995,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="2111" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2111" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2111">
         <v>7891024183083</v>
       </c>
@@ -58082,7 +58078,7 @@
         <v>4477</v>
       </c>
     </row>
-    <row r="2115" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2115" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2115">
         <v>7891040003167</v>
       </c>
@@ -58145,7 +58141,7 @@
         <v>4480</v>
       </c>
     </row>
-    <row r="2118" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2118" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2118">
         <v>7891050004741</v>
       </c>
@@ -58208,7 +58204,7 @@
         <v>4490</v>
       </c>
     </row>
-    <row r="2121" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2121" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2121">
         <v>7891079012895</v>
       </c>
@@ -59191,7 +59187,7 @@
         <v>4595</v>
       </c>
     </row>
-    <row r="2170" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2170" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2170">
         <v>8445290057433</v>
       </c>
@@ -59214,7 +59210,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="2171" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2171" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2171">
         <v>8445290067401</v>
       </c>
@@ -59257,7 +59253,7 @@
         <v>4380</v>
       </c>
     </row>
-    <row r="2173" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2173" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2173">
         <v>8445290068682</v>
       </c>
@@ -59420,7 +59416,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="2181" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2181" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2181">
         <v>8445290533982</v>
       </c>
@@ -59443,7 +59439,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="2182" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2182" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2182">
         <v>8445290584984</v>
       </c>
@@ -59466,7 +59462,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="2183" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2183" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2183">
         <v>8445290585004</v>
       </c>
@@ -59509,7 +59505,7 @@
         <v>4625</v>
       </c>
     </row>
-    <row r="2185" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2185" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2185">
         <v>8445290585240</v>
       </c>
@@ -59532,7 +59528,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="2186" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2186" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2186">
         <v>8445290615916</v>
       </c>
@@ -59555,7 +59551,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="2187" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2187" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2187">
         <v>8445290667571</v>
       </c>
@@ -59658,7 +59654,7 @@
         <v>4645</v>
       </c>
     </row>
-    <row r="2192" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2192" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2192">
         <v>8445290944429</v>
       </c>
@@ -59681,7 +59677,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="2193" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2193" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2193">
         <v>8445290944559</v>
       </c>
@@ -59724,7 +59720,7 @@
         <v>4645</v>
       </c>
     </row>
-    <row r="2195" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2195" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2195">
         <v>8445290977373</v>
       </c>
@@ -59767,7 +59763,7 @@
         <v>4645</v>
       </c>
     </row>
-    <row r="2197" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2197" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2197">
         <v>8445290986559</v>
       </c>
@@ -59790,7 +59786,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="2198" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2198" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2198">
         <v>8445290987587</v>
       </c>
@@ -59973,7 +59969,7 @@
         <v>4224</v>
       </c>
     </row>
-    <row r="2207" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2207" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2207">
         <v>8445291121904</v>
       </c>
@@ -60056,7 +60052,7 @@
         <v>4224</v>
       </c>
     </row>
-    <row r="2211" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2211" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2211">
         <v>8445291462830</v>
       </c>
@@ -60079,7 +60075,7 @@
         <v>4703</v>
       </c>
     </row>
-    <row r="2212" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2212" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2212">
         <v>8445291478923</v>
       </c>

</xml_diff>